<commit_message>
Throttling, crone joba and execution timeout added
</commit_message>
<xml_diff>
--- a/backend/public/excelsheets/order-chart.xlsx
+++ b/backend/public/excelsheets/order-chart.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C14"/>
+  <dimension ref="A1:C4"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
@@ -413,21 +413,21 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="1">
-        <v>45101.77083333333</v>
+        <v>45158.77083333333</v>
       </c>
       <c r="B2">
-        <v>12350</v>
+        <v>21996</v>
       </c>
       <c r="C2">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="1">
-        <v>45104.77083333333</v>
+        <v>45161.77083333333</v>
       </c>
       <c r="B3">
-        <v>1220</v>
+        <v>43500</v>
       </c>
       <c r="C3">
         <v>1</v>
@@ -435,123 +435,13 @@
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="1">
-        <v>45106.77083333333</v>
+        <v>45165.77083333333</v>
       </c>
       <c r="B4">
-        <v>15430</v>
+        <v>43500</v>
       </c>
       <c r="C4">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A5" s="1">
-        <v>45121.77083333333</v>
-      </c>
-      <c r="B5">
-        <v>22020</v>
-      </c>
-      <c r="C5">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A6" s="1">
-        <v>45127.77083333333</v>
-      </c>
-      <c r="B6">
-        <v>45000</v>
-      </c>
-      <c r="C6">
         <v>1</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A7" s="1">
-        <v>45131.77083333333</v>
-      </c>
-      <c r="B7">
-        <v>18500</v>
-      </c>
-      <c r="C7">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A8" s="1">
-        <v>45132.77083333333</v>
-      </c>
-      <c r="B8">
-        <v>14050</v>
-      </c>
-      <c r="C8">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A9" s="1">
-        <v>45134.77083333333</v>
-      </c>
-      <c r="B9">
-        <v>15990</v>
-      </c>
-      <c r="C9">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A10" s="1">
-        <v>45137.77083333333</v>
-      </c>
-      <c r="B10">
-        <v>60810</v>
-      </c>
-      <c r="C10">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A11" s="1">
-        <v>45140.77083333333</v>
-      </c>
-      <c r="B11">
-        <v>3979</v>
-      </c>
-      <c r="C11">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A12" s="1">
-        <v>45141.77083333333</v>
-      </c>
-      <c r="B12">
-        <v>34190</v>
-      </c>
-      <c r="C12">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A13" s="1">
-        <v>45145.77083333333</v>
-      </c>
-      <c r="B13">
-        <v>2370</v>
-      </c>
-      <c r="C13">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A14" s="1">
-        <v>45146.77083333333</v>
-      </c>
-      <c r="B14">
-        <v>3800</v>
-      </c>
-      <c r="C14">
-        <v>2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>